<commit_message>
Polish native Excel Pareto chart styling
Rebuild the in-workbook Pareto chart: per-bar colors highlighting the
vital few (deep blue) vs tail (light blue), value data labels, styled
cumulative line with % labels, dashed 80% target line, rotated category
names, light gridlines, and a styled title/axes. Regenerate preview PNGs
to match the native chart design.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzhegtSCJ2gUncrSCG1F8E
</commit_message>
<xml_diff>
--- a/pelvic-block-iqc-pareto/Pelvic_Block_IQC_Pareto_RootCause.xlsx
+++ b/pelvic-block-iqc-pareto/Pelvic_Block_IQC_Pareto_RootCause.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -101,6 +101,12 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -242,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -298,6 +304,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -333,58 +340,58 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="1" fontId="18" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="18" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -463,7 +470,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -471,14 +477,26 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Defect Pareto — Rejected Pelvic Blocks (SH: Martins, 2026-07-08)</a:t>
+              <a:rPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Defect Pareto — Rejected Pelvic Blocks   (SH: Martins, 2026-07-08)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -493,13 +511,183 @@
             </strRef>
           </tx>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E5B8A"/>
+            </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E5B8A"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E5B8A"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E5B8A"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E5B8A"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="4"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="AFC7E3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="5"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="AFC7E3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="AFC7E3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="7"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="AFC7E3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="8"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="AFC7E3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="9"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="AFC7E3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dLbls>
+            <numFmt formatCode="0"/>
+            <txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="950" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="404040"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="950" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="404040"/>
+                  </a:solidFill>
+                  <a:latin typeface="Calibri"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showVal val="1"/>
+          </dLbls>
           <cat>
             <numRef>
-              <f>'Pareto'!$C$6:$C$15</f>
+              <f>'Pareto'!$M$6:$M$15</f>
             </numRef>
           </cat>
           <val>
@@ -508,7 +696,7 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="40"/>
+        <gapWidth val="55"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -523,13 +711,80 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln w="28575">
+              <a:solidFill>
+                <a:srgbClr val="C0504D"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="circle"/>
-            <size val="5"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="C0504D"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <numFmt formatCode="0%"/>
+            <txPr>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="850" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="C0504D"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="850" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="C0504D"/>
+                  </a:solidFill>
+                  <a:latin typeface="Calibri"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="t"/>
+            <showVal val="1"/>
+          </dLbls>
+          <val>
+            <numRef>
+              <f>'Pareto'!$F$6:$F$15</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Pareto'!N5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="A6A6A6"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -538,7 +793,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Pareto'!$F$6:$F$15</f>
+              <f>'Pareto'!$N$6:$N$15</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -551,24 +806,40 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Defect mode</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <spPr>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="BFBFBF"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-2700000"/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="850" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="595959"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="850" b="0">
+              <a:solidFill>
+                <a:srgbClr val="595959"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -576,9 +847,20 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E6E6E6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
         <title>
           <tx>
             <rich>
@@ -594,8 +876,31 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="595959"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="595959"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
         <crosses val="autoZero"/>
       </valAx>
@@ -606,8 +911,8 @@
           <max val="1"/>
           <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
         <title>
           <tx>
             <rich>
@@ -626,12 +931,35 @@
         <numFmt formatCode="0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="595959"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="595959"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
         <crosses val="max"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
+      <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -648,7 +976,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="4320000"/>
+    <ext cx="9360000" cy="4500000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -665,12 +993,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>0</col>
       <colOff>0</colOff>
       <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6819900" cy="3114675"/>
+    <ext cx="5667375" cy="2905125"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -3734,7 +4062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3797,17 +4125,23 @@
           <t>Cumulative %</t>
         </is>
       </c>
+      <c r="M5" s="19" t="n"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>80% target</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="A6" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Membrane damage in critical area</t>
         </is>
@@ -3816,25 +4150,33 @@
         <f>SUM('Inspection Log'!Q5:Q430)</f>
         <v/>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="23">
         <f>D6/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="23">
         <f>E6</f>
         <v/>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>D6 · Membrane dmg</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>Ureters not embedded</t>
         </is>
@@ -3843,25 +4185,33 @@
         <f>SUM('Inspection Log'!L5:L430)</f>
         <v/>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="23">
         <f>D7/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="23">
         <f>F6+E7</f>
         <v/>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>D1 · Ureters n/e</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n">
+      <c r="A8" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Suspensory ligaments damaged</t>
         </is>
@@ -3870,25 +4220,33 @@
         <f>SUM('Inspection Log'!O5:O430)</f>
         <v/>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="23">
         <f>D8/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="23">
         <f>F7+E8</f>
         <v/>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>D4 · Susp. ligament</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>Urethra cut</t>
         </is>
@@ -3897,25 +4255,33 @@
         <f>SUM('Inspection Log'!P5:P430)</f>
         <v/>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="23">
         <f>D9/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="23">
         <f>F8+E9</f>
         <v/>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>D5 · Urethra cut</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n">
+      <c r="A10" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>Ureter missing</t>
         </is>
@@ -3924,25 +4290,33 @@
         <f>SUM('Inspection Log'!N5:N430)</f>
         <v/>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="23">
         <f>D10/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="23">
         <f>F9+E10</f>
         <v/>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>D3 · Ureter missing</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n">
+      <c r="A11" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>Bowel cut / opened / separated</t>
         </is>
@@ -3951,25 +4325,33 @@
         <f>SUM('Inspection Log'!S5:S430)</f>
         <v/>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="23">
         <f>D11/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="23">
         <f>F10+E11</f>
         <v/>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>D8 · Bowel cut</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n">
+      <c r="A12" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>Ureter cut / severed</t>
         </is>
@@ -3978,25 +4360,33 @@
         <f>SUM('Inspection Log'!M5:M430)</f>
         <v/>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="23">
         <f>D12/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="23">
         <f>F11+E12</f>
         <v/>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>D2 · Ureter cut</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n">
+      <c r="A13" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>Bladder deformed / deformed attachment</t>
         </is>
@@ -4005,25 +4395,33 @@
         <f>SUM('Inspection Log'!R5:R430)</f>
         <v/>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="23">
         <f>D13/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="23">
         <f>F12+E13</f>
         <v/>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>D7 · Bladder def.</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n">
+      <c r="A14" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
+      <c r="C14" s="24" t="inlineStr">
         <is>
           <t>Blood clots</t>
         </is>
@@ -4032,25 +4430,33 @@
         <f>SUM('Inspection Log'!T5:T430)</f>
         <v/>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="23">
         <f>D14/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="23">
         <f>F13+E14</f>
         <v/>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>D9 · Blood clots</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n">
+      <c r="A15" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="24" t="inlineStr">
         <is>
           <t>Broad ligament hole / tear</t>
         </is>
@@ -4059,32 +4465,40 @@
         <f>SUM('Inspection Log'!U5:U430)</f>
         <v/>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="23">
         <f>D15/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="23">
         <f>F14+E15</f>
         <v/>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>D10 · Broad ligament</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="n"/>
-      <c r="B16" s="24" t="n"/>
-      <c r="C16" s="25" t="inlineStr">
+      <c r="A16" s="25" t="n"/>
+      <c r="B16" s="25" t="n"/>
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="27">
         <f>SUM(D6:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="27">
+      <c r="E16" s="28">
         <f>D16/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="F16" s="24" t="n"/>
+      <c r="F16" s="25" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr">
@@ -4121,37 +4535,37 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="B21" s="29" t="inlineStr">
+      <c r="B21" s="30" t="inlineStr">
         <is>
           <t>Evisceration</t>
         </is>
       </c>
-      <c r="C21" s="30">
+      <c r="C21" s="31">
         <f>SUM('Inspection Log'!L5:L430)+SUM('Inspection Log'!M5:M430)+SUM('Inspection Log'!O5:O430)+SUM('Inspection Log'!Q5:Q430)+SUM('Inspection Log'!S5:S430)+SUM('Inspection Log'!U5:U430)</f>
         <v/>
       </c>
-      <c r="D21" s="31">
+      <c r="D21" s="32">
         <f>C21/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="E21" s="29" t="inlineStr">
+      <c r="E21" s="30" t="inlineStr">
         <is>
           <t>D1, D2, D4, D6, D8, D10</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="B22" s="23" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Carcass splitting</t>
         </is>
@@ -4160,23 +4574,23 @@
         <f>SUM('Inspection Log'!P5:P430)</f>
         <v/>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="23">
         <f>C22/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="E22" s="23" t="inlineStr">
+      <c r="E22" s="24" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>Bung dropping</t>
         </is>
@@ -4185,23 +4599,23 @@
         <f>SUM('Inspection Log'!N5:N430)</f>
         <v/>
       </c>
-      <c r="D23" s="22">
+      <c r="D23" s="23">
         <f>C23/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="E23" s="23" t="inlineStr">
+      <c r="E23" s="24" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="B24" s="24" t="inlineStr">
         <is>
           <t>Live / physiology</t>
         </is>
@@ -4210,23 +4624,23 @@
         <f>SUM('Inspection Log'!R5:R430)</f>
         <v/>
       </c>
-      <c r="D24" s="22">
+      <c r="D24" s="23">
         <f>C24/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="E24" s="23" t="inlineStr">
+      <c r="E24" s="24" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="24" t="inlineStr">
         <is>
           <t>Sticking / Bleeding</t>
         </is>
@@ -4235,11 +4649,11 @@
         <f>SUM('Inspection Log'!T5:T430)</f>
         <v/>
       </c>
-      <c r="D25" s="22">
+      <c r="D25" s="23">
         <f>C25/SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
-      <c r="E25" s="23" t="inlineStr">
+      <c r="E25" s="24" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
@@ -4362,53 +4776,53 @@
           <t>D6</t>
         </is>
       </c>
-      <c r="B5" s="32" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>Membrane damage in critical area</t>
         </is>
       </c>
-      <c r="C5" s="33" t="inlineStr">
+      <c r="C5" s="34" t="inlineStr">
         <is>
           <t>Membrane torn/holed in critical area</t>
         </is>
       </c>
-      <c r="D5" s="33" t="inlineStr">
+      <c r="D5" s="34" t="inlineStr">
         <is>
           <t>Knife path too deep / tensile tear during gut pull</t>
         </is>
       </c>
-      <c r="E5" s="33" t="inlineStr">
+      <c r="E5" s="34" t="inlineStr">
         <is>
           <t>Evisceration technique not standardized for pelvic zone</t>
         </is>
       </c>
-      <c r="F5" s="33" t="inlineStr">
+      <c r="F5" s="34" t="inlineStr">
         <is>
           <t>No defined knife depth/path SOP + line speed pressure</t>
         </is>
       </c>
-      <c r="G5" s="34" t="inlineStr">
+      <c r="G5" s="35" t="inlineStr">
         <is>
           <t>(confirm w/ supplier) training + line-speed control gap</t>
         </is>
       </c>
-      <c r="H5" s="35" t="inlineStr">
+      <c r="H5" s="36" t="inlineStr">
         <is>
           <t>Retrain knife depth &amp; path in pelvic zone; blunt-dissect; slow line through pelvic cut</t>
         </is>
       </c>
-      <c r="I5" s="36" t="inlineStr">
+      <c r="I5" s="37" t="inlineStr">
         <is>
           <t>SH Martins - Evisceration lead</t>
         </is>
       </c>
-      <c r="J5" s="36" t="inlineStr"/>
-      <c r="K5" s="37" t="inlineStr">
+      <c r="J5" s="37" t="inlineStr"/>
+      <c r="K5" s="38" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="L5" s="38" t="inlineStr"/>
+      <c r="L5" s="39" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
@@ -4416,53 +4830,53 @@
           <t>D1</t>
         </is>
       </c>
-      <c r="B6" s="32" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>Ureters not embedded</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="34" t="inlineStr">
         <is>
           <t>Ureters not embedded in tissue</t>
         </is>
       </c>
-      <c r="D6" s="33" t="inlineStr">
+      <c r="D6" s="34" t="inlineStr">
         <is>
           <t>Fascia/perirenal fat stripped away from ureter</t>
         </is>
       </c>
-      <c r="E6" s="33" t="inlineStr">
+      <c r="E6" s="34" t="inlineStr">
         <is>
           <t>Excessive pull force / over-trim during gut set removal</t>
         </is>
       </c>
-      <c r="F6" s="33" t="inlineStr">
+      <c r="F6" s="34" t="inlineStr">
         <is>
           <t>Pull technique &amp; trim spec not controlled</t>
         </is>
       </c>
-      <c r="G6" s="34" t="inlineStr">
+      <c r="G6" s="35" t="inlineStr">
         <is>
           <t>(confirm) handling standard missing</t>
         </is>
       </c>
-      <c r="H6" s="35" t="inlineStr">
+      <c r="H6" s="36" t="inlineStr">
         <is>
           <t>Standardize pull-force &amp; angle; limit fat stripping; gentler pit drop</t>
         </is>
       </c>
-      <c r="I6" s="36" t="inlineStr">
+      <c r="I6" s="37" t="inlineStr">
         <is>
           <t>SH Martins - Evisceration lead</t>
         </is>
       </c>
-      <c r="J6" s="36" t="inlineStr"/>
-      <c r="K6" s="37" t="inlineStr">
+      <c r="J6" s="37" t="inlineStr"/>
+      <c r="K6" s="38" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="L6" s="38" t="inlineStr"/>
+      <c r="L6" s="39" t="inlineStr"/>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
@@ -4470,53 +4884,53 @@
           <t>D4</t>
         </is>
       </c>
-      <c r="B7" s="32" t="inlineStr">
+      <c r="B7" s="33" t="inlineStr">
         <is>
           <t>Suspensory ligaments damaged</t>
         </is>
       </c>
-      <c r="C7" s="33" t="inlineStr">
+      <c r="C7" s="34" t="inlineStr">
         <is>
           <t>Suspensory ligaments torn/frayed</t>
         </is>
       </c>
-      <c r="D7" s="33" t="inlineStr">
+      <c r="D7" s="34" t="inlineStr">
         <is>
           <t>Block pulled/handled by the ligaments</t>
         </is>
       </c>
-      <c r="E7" s="33" t="inlineStr">
+      <c r="E7" s="34" t="inlineStr">
         <is>
           <t>Rough handling + high traction on removal</t>
         </is>
       </c>
-      <c r="F7" s="33" t="inlineStr">
+      <c r="F7" s="34" t="inlineStr">
         <is>
           <t>No 'support-surface' handling rule</t>
         </is>
       </c>
-      <c r="G7" s="34" t="inlineStr">
+      <c r="G7" s="35" t="inlineStr">
         <is>
           <t>(confirm) handling standard missing</t>
         </is>
       </c>
-      <c r="H7" s="35" t="inlineStr">
+      <c r="H7" s="36" t="inlineStr">
         <is>
           <t>Handle block by support surface, not ligaments; control pull force</t>
         </is>
       </c>
-      <c r="I7" s="36" t="inlineStr">
+      <c r="I7" s="37" t="inlineStr">
         <is>
           <t>SH Martins - Evisceration lead</t>
         </is>
       </c>
-      <c r="J7" s="36" t="inlineStr"/>
-      <c r="K7" s="37" t="inlineStr">
+      <c r="J7" s="37" t="inlineStr"/>
+      <c r="K7" s="38" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="L7" s="38" t="inlineStr"/>
+      <c r="L7" s="39" t="inlineStr"/>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
@@ -4524,53 +4938,53 @@
           <t>D5</t>
         </is>
       </c>
-      <c r="B8" s="32" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>Urethra cut</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="C8" s="34" t="inlineStr">
         <is>
           <t>Urethra cut</t>
         </is>
       </c>
-      <c r="D8" s="33" t="inlineStr">
+      <c r="D8" s="34" t="inlineStr">
         <is>
           <t>Sharp transection through pelvic zone</t>
         </is>
       </c>
-      <c r="E8" s="33" t="inlineStr">
+      <c r="E8" s="34" t="inlineStr">
         <is>
           <t>Splitting saw off-center / bung-drop cut catches urethra</t>
         </is>
       </c>
-      <c r="F8" s="33" t="inlineStr">
+      <c r="F8" s="34" t="inlineStr">
         <is>
           <t>Saw alignment &amp; pelvic-split centering not verified</t>
         </is>
       </c>
-      <c r="G8" s="34" t="inlineStr">
+      <c r="G8" s="35" t="inlineStr">
         <is>
           <t>(confirm) saw calibration + technique gap</t>
         </is>
       </c>
-      <c r="H8" s="35" t="inlineStr">
+      <c r="H8" s="36" t="inlineStr">
         <is>
           <t>Center split on symphysis; calibrate/align saw; slow through pelvic zone</t>
         </is>
       </c>
-      <c r="I8" s="36" t="inlineStr">
+      <c r="I8" s="37" t="inlineStr">
         <is>
           <t>SH Martins - Splitting lead</t>
         </is>
       </c>
-      <c r="J8" s="36" t="inlineStr"/>
-      <c r="K8" s="37" t="inlineStr">
+      <c r="J8" s="37" t="inlineStr"/>
+      <c r="K8" s="38" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="L8" s="38" t="inlineStr"/>
+      <c r="L8" s="39" t="inlineStr"/>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
@@ -4578,81 +4992,81 @@
           <t>D8</t>
         </is>
       </c>
-      <c r="B9" s="32" t="inlineStr">
+      <c r="B9" s="33" t="inlineStr">
         <is>
           <t>Bowel cut / opened / separated</t>
         </is>
       </c>
-      <c r="C9" s="33" t="inlineStr">
+      <c r="C9" s="34" t="inlineStr">
         <is>
           <t>Bowel cut open / separated (FOOD SAFETY)</t>
         </is>
       </c>
-      <c r="D9" s="33" t="inlineStr">
+      <c r="D9" s="34" t="inlineStr">
         <is>
           <t>Knife slip or aggressive bung separation opens bowel</t>
         </is>
       </c>
-      <c r="E9" s="33" t="inlineStr">
+      <c r="E9" s="34" t="inlineStr">
         <is>
           <t>Bung not adequately bagged/tied before cut</t>
         </is>
       </c>
-      <c r="F9" s="33" t="inlineStr">
+      <c r="F9" s="34" t="inlineStr">
         <is>
           <t>Bung-dropping CCP not robust</t>
         </is>
       </c>
-      <c r="G9" s="34" t="inlineStr">
+      <c r="G9" s="35" t="inlineStr">
         <is>
           <t>(confirm) contamination-control gap at bung station</t>
         </is>
       </c>
-      <c r="H9" s="35" t="inlineStr">
+      <c r="H9" s="36" t="inlineStr">
         <is>
           <t>Reinforce bung bag/tie-off; retrain knife path; treat as contamination CCP</t>
         </is>
       </c>
-      <c r="I9" s="36" t="inlineStr">
+      <c r="I9" s="37" t="inlineStr">
         <is>
           <t>SH Martins - Bung/Evisc. lead</t>
         </is>
       </c>
-      <c r="J9" s="36" t="inlineStr"/>
-      <c r="K9" s="37" t="inlineStr">
+      <c r="J9" s="37" t="inlineStr"/>
+      <c r="K9" s="38" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="L9" s="38" t="inlineStr"/>
+      <c r="L9" s="39" t="inlineStr"/>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="39" t="n"/>
-      <c r="B10" s="39" t="n"/>
-      <c r="C10" s="39" t="n"/>
-      <c r="D10" s="39" t="n"/>
-      <c r="E10" s="39" t="n"/>
-      <c r="F10" s="39" t="n"/>
-      <c r="G10" s="40" t="n"/>
-      <c r="H10" s="41" t="n"/>
-      <c r="I10" s="39" t="n"/>
-      <c r="J10" s="39" t="n"/>
-      <c r="K10" s="39" t="n"/>
-      <c r="L10" s="42" t="n"/>
+      <c r="A10" s="40" t="n"/>
+      <c r="B10" s="40" t="n"/>
+      <c r="C10" s="40" t="n"/>
+      <c r="D10" s="40" t="n"/>
+      <c r="E10" s="40" t="n"/>
+      <c r="F10" s="40" t="n"/>
+      <c r="G10" s="41" t="n"/>
+      <c r="H10" s="42" t="n"/>
+      <c r="I10" s="40" t="n"/>
+      <c r="J10" s="40" t="n"/>
+      <c r="K10" s="40" t="n"/>
+      <c r="L10" s="43" t="n"/>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="39" t="n"/>
-      <c r="B11" s="39" t="n"/>
-      <c r="C11" s="39" t="n"/>
-      <c r="D11" s="39" t="n"/>
-      <c r="E11" s="39" t="n"/>
-      <c r="F11" s="39" t="n"/>
-      <c r="G11" s="40" t="n"/>
-      <c r="H11" s="41" t="n"/>
-      <c r="I11" s="39" t="n"/>
-      <c r="J11" s="39" t="n"/>
-      <c r="K11" s="39" t="n"/>
-      <c r="L11" s="42" t="n"/>
+      <c r="A11" s="40" t="n"/>
+      <c r="B11" s="40" t="n"/>
+      <c r="C11" s="40" t="n"/>
+      <c r="D11" s="40" t="n"/>
+      <c r="E11" s="40" t="n"/>
+      <c r="F11" s="40" t="n"/>
+      <c r="G11" s="41" t="n"/>
+      <c r="H11" s="42" t="n"/>
+      <c r="I11" s="40" t="n"/>
+      <c r="J11" s="40" t="n"/>
+      <c r="K11" s="40" t="n"/>
+      <c r="L11" s="43" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4700,119 +5114,119 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="43" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>KEY METRICS</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="44" t="inlineStr">
+      <c r="A5" s="45" t="inlineStr">
         <is>
           <t>Blocks Inspected</t>
         </is>
       </c>
-      <c r="B5" s="45">
+      <c r="B5" s="46">
         <f>COUNTA('Inspection Log'!A5:A430)-COUNTBLANK('Inspection Log'!A5:A430)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="A6" s="45" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="B6" s="45">
+      <c r="B6" s="46">
         <f>COUNTIF('Inspection Log'!J5:J430,"Pass")</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="44" t="inlineStr">
+      <c r="A7" s="45" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="B7" s="45">
+      <c r="B7" s="46">
         <f>COUNTIF('Inspection Log'!J5:J430,"Fail")</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="44" t="inlineStr">
+      <c r="A8" s="45" t="inlineStr">
         <is>
           <t>First Pass Yield</t>
         </is>
       </c>
-      <c r="B8" s="46">
+      <c r="B8" s="47">
         <f>IFERROR(COUNTIF('Inspection Log'!J5:J430,"Pass")/(COUNTA('Inspection Log'!A5:A430)-COUNTBLANK('Inspection Log'!A5:A430)),0)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="44" t="inlineStr">
+      <c r="A9" s="45" t="inlineStr">
         <is>
           <t>Total Defect Occurrences</t>
         </is>
       </c>
-      <c r="B9" s="45">
+      <c r="B9" s="46">
         <f>SUM('Inspection Log'!L5:U430)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="44" t="inlineStr">
+      <c r="A10" s="45" t="inlineStr">
         <is>
           <t>Defects per Failed Block</t>
         </is>
       </c>
-      <c r="B10" s="47">
+      <c r="B10" s="48">
         <f>IFERROR(SUM('Inspection Log'!L5:U430)/COUNTIF('Inspection Log'!J5:J430,"Fail"),0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="43" t="inlineStr">
+      <c r="A12" s="44" t="inlineStr">
         <is>
           <t>TOP DEFECT (this batch)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="48" t="inlineStr">
+      <c r="A13" s="49" t="inlineStr">
         <is>
           <t>Membrane damage in critical area</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="49" t="inlineStr">
+      <c r="A14" s="50" t="inlineStr">
         <is>
           <t>Dominant supplier station</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="50" t="inlineStr">
+      <c r="A15" s="51" t="inlineStr">
         <is>
           <t>S3 Evisceration  -&gt;  primary target for corrective action</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="51" t="inlineStr">
+      <c r="A17" s="52" t="inlineStr">
         <is>
           <t>Critical / food-safety defect occurrences</t>
         </is>
       </c>
-      <c r="B17" s="52">
+      <c r="B17" s="53">
         <f>SUM('Inspection Log'!Q5:Q430)+SUM('Inspection Log'!S5:S430)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="53" t="inlineStr">
+      <c r="A18" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Critical codes: D6, D8 — membrane damage &amp; bowel breach)</t>
         </is>

</xml_diff>

<commit_message>
Fix and declutter the Pareto chart
Excel was rendering the data labels as 'Count, D6 · Membrane dmg, 49'
because only showVal was set; explicitly disable series/category/legend
name flags so bars show value only. Remove the per-point labels from the
cumulative line (the exact %s are already in the Pareto table) and thin
the line so it reads as a subtle reference rather than clutter.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzhegtSCJ2gUncrSCG1F8E
</commit_message>
<xml_diff>
--- a/pelvic-block-iqc-pareto/Pelvic_Block_IQC_Pareto_RootCause.xlsx
+++ b/pelvic-block-iqc-pareto/Pelvic_Block_IQC_Pareto_RootCause.xlsx
@@ -723,7 +723,7 @@
               <a:bodyPr/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="950" b="1">
+                  <a:defRPr sz="1000" b="1">
                     <a:solidFill>
                       <a:srgbClr val="404040"/>
                     </a:solidFill>
@@ -733,7 +733,7 @@
                 <a:r>
                   <a:t/>
                 </a:r>
-                <a:endParaRPr sz="950" b="1">
+                <a:endParaRPr sz="1000" b="1">
                   <a:solidFill>
                     <a:srgbClr val="404040"/>
                   </a:solidFill>
@@ -742,7 +742,12 @@
               </a:p>
             </txPr>
             <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
             <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
           </dLbls>
           <cat>
             <numRef>
@@ -770,7 +775,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="28575">
+            <a:ln w="19050">
               <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
@@ -779,7 +784,7 @@
           </spPr>
           <marker>
             <symbol val="circle"/>
-            <size val="6"/>
+            <size val="5"/>
             <spPr>
               <a:solidFill>
                 <a:srgbClr val="C0504D"/>
@@ -793,31 +798,12 @@
             </spPr>
           </marker>
           <dLbls>
-            <numFmt formatCode="0%"/>
-            <txPr>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="850" b="1">
-                    <a:solidFill>
-                      <a:srgbClr val="C0504D"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-                <a:endParaRPr sz="850" b="1">
-                  <a:solidFill>
-                    <a:srgbClr val="C0504D"/>
-                  </a:solidFill>
-                  <a:latin typeface="Calibri"/>
-                </a:endParaRPr>
-              </a:p>
-            </txPr>
-            <dLblPos val="t"/>
-            <showVal val="1"/>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
           </dLbls>
           <val>
             <numRef>
@@ -850,6 +836,14 @@
               </a:ln>
             </spPr>
           </marker>
+          <dLbls>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+          </dLbls>
           <val>
             <numRef>
               <f>'Pareto'!$N$6:$N$18</f>

</xml_diff>

<commit_message>
Add Yield & Alignment sheet (good-pelvic % + tech/inspector alignment)
New 'Yield & Alignment' sheet: headline good-pelvic rate across the
board (10.1% = 10/99), a good-rate breakdown by inspection sheet
(kill date x inspector, via COUNTIFS), an interpretation of what a
~10% yield may mean for harvest-tech training (material vs calibration
gap), and a tech<->inspector alignment section. Alignment is framed
honestly: we can only observe agreement on KEPT blocks (~10%) today,
confounded with material quality, so input cells are provided to enter
the techs' first-pass discard counts and compute true alignment going
forward. Adds Yield_snapshot.png.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzhegtSCJ2gUncrSCG1F8E
</commit_message>
<xml_diff>
--- a/pelvic-block-iqc-pareto/Pelvic_Block_IQC_Pareto_RootCause.xlsx
+++ b/pelvic-block-iqc-pareto/Pelvic_Block_IQC_Pareto_RootCause.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Root-Cause Deep-Dive" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Root Cause 5-Why" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Dashboard" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Yield &amp; Alignment" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -197,6 +198,23 @@
       <color rgb="00833C00"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="40"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00444444"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -316,7 +334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -482,6 +500,36 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="29" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1434,7 +1482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1562,107 +1610,115 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7. Yield &amp; Alignment   Good-pelvic % across the board; what it may mean for harvest-tech training; and tech&lt;-&gt;inspector alignment (with input cells).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>HOW TO ADD THE NEXT INSPECTION</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  a. In 'Inspection Log', add one row per inspected block (metadata + Result = Pass/Fail + verbatim reason).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  b. Put a 1 in each defect column (D1–D11) that applies. Use the dropdown. If a NEW defect type appears, add it to 'Defect Taxonomy' first, then add its column.</t>
+          <t xml:space="preserve">  a. In 'Inspection Log', add one row per inspected block (metadata + Result = Pass/Fail + verbatim reason).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  b. Put a 1 in each defect column (D1–D11) that applies. Use the dropdown. If a NEW defect type appears, add it to 'Defect Taxonomy' first, then add its column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  c. Pareto + Dashboard recalc automatically. Re-sort the Pareto table high-&gt;low if the ranking changes (counts are live; row order is not).</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>WHAT THE DATA SAYS SO FAR  (4 inspection sheets across 3 kill dates: 2026-05-27, 2026-07-08, 2026-07-28 — SH: Martins)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  99 blocks inspected · 10 pass · 89 fail · combined First Pass Yield 10.1% · 122 defect occurrences</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Vital few (~80%): membrane damage (critical area), ureters not embedded, urethra breach, bowel/colon/rectum breach, suspensory-ligament damage.  ~84% of ALL defects originate at ONE station: Evisceration.</t>
+          <t xml:space="preserve">  99 blocks inspected · 10 pass · 89 fail · combined First Pass Yield 10.1% · 122 defect occurrences</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Vital few (~80%): membrane damage (critical area), ureters not embedded, urethra breach, bowel/colon/rectum breach, suspensory-ligament damage.  ~84% of ALL defects originate at ONE station: Evisceration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  OPEN ITEMS: (1) 5 blocks (kill 2026-05-27), 8" hole in bladder suspensory ligament — recorded PASS pending ME/DE (flip to Fail + tag D4 if confirmed).  (2) Rasmin 07-28 sheet handwritten total said '22 fails' but per-row entries sum to 29 (used).</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>SEVERITY KEY</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  Critical = function-destroying or food-safety (e.g. bowel/colon/rectum breach = contamination).   Major = block rejected.   Minor = cosmetic / recoverable.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr"/>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>SOURCE</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  IQC Tally Sheets — SH: Martins. Originals kept as source_*.xlsx in this folder.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="35">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A30:H30"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A6:H6"/>
@@ -11861,4 +11917,429 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>YIELD &amp; INSPECTOR–TECH ALIGNMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>How many pelvics are good across the board — and what it may say about harvest-tech training and tech&lt;-&gt;inspector alignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>GOOD PELVICS — ACROSS THE BOARD  (First Pass Yield = good / inspected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="65">
+        <f>IFERROR(COUNTIFS('Inspection Log'!J5:J503,"Pass")/(COUNTIFS('Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!J5:J503,"Fail")),0)</f>
+        <v/>
+      </c>
+      <c r="B5" s="51" t="n"/>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>of pelvic blocks that reach inspection pass IQC on the first look.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="51" t="n"/>
+      <c r="B6" s="51" t="n"/>
+      <c r="C6" s="67">
+        <f>"= "&amp;COUNTIFS('Inspection Log'!J5:J503,"Pass")&amp;" good  /  "&amp;(COUNTIFS('Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!J5:J503,"Fail"))&amp;" inspected  -&gt;  ~9 of every 10 blocks are rejected"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="51" t="n"/>
+      <c r="B7" s="51" t="n"/>
+      <c r="C7" s="68" t="inlineStr">
+        <is>
+          <t>A yield this low is first a SUPPLIER signal (84% of defects are evisceration-origin) — but it also frames the tech/inspector questions below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="69" t="inlineStr">
+        <is>
+          <t>Caveat: the 8 passes on 2026-05-27 include 5 blocks recorded Pass pending ME/DE. If those are confirmed failures, the across-the-board good rate falls to ~5% (5/99).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>GOOD RATE BY INSPECTION SHEET  (kill date x inspector)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Kill Date</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Inspector</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Inspected</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Good (pass)</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Good %</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>(unnamed)</t>
+        </is>
+      </c>
+      <c r="C12" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-05-27",'Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!C5:C503,"2026-05-27",'Inspection Log'!J5:J503,"Fail")</f>
+        <v/>
+      </c>
+      <c r="D12" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-05-27",'Inspection Log'!J5:J503,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E12" s="70">
+        <f>IFERROR(D12/C12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>(unnamed)</t>
+        </is>
+      </c>
+      <c r="C13" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-08",'Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!C5:C503,"2026-07-08",'Inspection Log'!J5:J503,"Fail")</f>
+        <v/>
+      </c>
+      <c r="D13" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-08",'Inspection Log'!J5:J503,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E13" s="70">
+        <f>IFERROR(D13/C13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Rasmin</t>
+        </is>
+      </c>
+      <c r="C14" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-28",'Inspection Log'!G5:G503,"Rasmin",'Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!C5:C503,"2026-07-28",'Inspection Log'!G5:G503,"Rasmin",'Inspection Log'!J5:J503,"Fail")</f>
+        <v/>
+      </c>
+      <c r="D14" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-28",'Inspection Log'!G5:G503,"Rasmin",'Inspection Log'!J5:J503,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E14" s="70">
+        <f>IFERROR(D14/C14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Toni</t>
+        </is>
+      </c>
+      <c r="C15" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-28",'Inspection Log'!G5:G503,"Toni",'Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!C5:C503,"2026-07-28",'Inspection Log'!G5:G503,"Toni",'Inspection Log'!J5:J503,"Fail")</f>
+        <v/>
+      </c>
+      <c r="D15" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-28",'Inspection Log'!G5:G503,"Toni",'Inspection Log'!J5:J503,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E15" s="70">
+        <f>IFERROR(D15/C15,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr"/>
+      <c r="C16" s="29">
+        <f>COUNTIFS('Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!J5:J503,"Fail")</f>
+        <v/>
+      </c>
+      <c r="D16" s="29">
+        <f>COUNTIFS('Inspection Log'!J5:J503,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E16" s="71">
+        <f>IFERROR(D16/C16,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>WHAT THIS COULD MEAN ABOUT HARVEST-TECH TRAINING</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="36" t="inlineStr">
+        <is>
+          <t>The harvest techs are the first-pass filter: they recover blocks from the pit and keep (spec-out) or discard each one. A ~10% good rate can mean two very different things, and the current data cannot fully separate them:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="72" t="inlineStr">
+        <is>
+          <t>1)  MATERIAL (most likely).  The incoming tissue is overwhelmingly defective — 84% of defects are evisceration-origin — so even a perfectly-trained tech would keep mostly-bad blocks because there is little good material to choose from. Here the low yield is a SUPPLIER signal, not a tech signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="72" t="inlineStr">
+        <is>
+          <t>2)  CALIBRATION GAP.  If the techs are keeping blocks that inspectors then reject, their internal 'good/bad' threshold is looser than the inspection spec — a training / standardization gap. The tell for this is a high tech KEEP rate paired with a low IQC pass rate (see alignment below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="A22" s="73" t="inlineStr">
+        <is>
+          <t>Reading them together: because the defects are dominated by real, supplier-side damage, (1) is the stronger explanation today — but (2) cannot be ruled out until we log the techs' keep/discard decisions. A quick check: have a lead re-grade a sample of kept AND discarded blocks against the written spec and compare to both the tech and the inspector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>INSPECTOR &lt;-&gt; HARVEST-TECH ALIGNMENT  (agreement on the good/bad call)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="64" customHeight="1">
+      <c r="A25" s="36" t="inlineStr">
+        <is>
+          <t>Alignment = do the harvest tech (keep/discard) and the inspector (pass/fail) make the SAME good/bad call on the same block? What we can see now: the inspected blocks are the ones the techs KEPT, and inspectors pass only ~10% of them — so on the KEEP decision the two groups agree ~10% of the time (9 of 10 blocks a tech judged good enough to keep, the inspector rejected). That is a strong misalignment signal, but it is confounded with material quality, and we cannot yet see the techs' DISCARD calls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="73" t="inlineStr">
+        <is>
+          <t>To measure alignment properly, enter the harvest-tech first-pass numbers below (received from pit, discarded first-pass). Then the agreement metrics compute automatically. Also re-inspect a sample of discarded blocks to catch over-discarding (good blocks thrown away).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Kill Date</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Received from pit  (enter)</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Tech discarded 1st-pass  (enter)</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>IQC inspected (=kept)</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>IQC good</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Tech reject %</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Good-from-pit %</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B29" s="74" t="n"/>
+      <c r="C29" s="74" t="n"/>
+      <c r="D29" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-05-27",'Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!C5:C503,"2026-05-27",'Inspection Log'!J5:J503,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E29" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-05-27",'Inspection Log'!J5:J503,"Pass")</f>
+        <v/>
+      </c>
+      <c r="F29" s="70">
+        <f>IF(B29="","",IFERROR(C29/B29,0))</f>
+        <v/>
+      </c>
+      <c r="G29" s="70">
+        <f>IF(B29="","",IFERROR(E29/B29,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B30" s="74" t="n"/>
+      <c r="C30" s="74" t="n"/>
+      <c r="D30" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-08",'Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!C5:C503,"2026-07-08",'Inspection Log'!J5:J503,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E30" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-08",'Inspection Log'!J5:J503,"Pass")</f>
+        <v/>
+      </c>
+      <c r="F30" s="70">
+        <f>IF(B30="","",IFERROR(C30/B30,0))</f>
+        <v/>
+      </c>
+      <c r="G30" s="70">
+        <f>IF(B30="","",IFERROR(E30/B30,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B31" s="74" t="n"/>
+      <c r="C31" s="74" t="n"/>
+      <c r="D31" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-28",'Inspection Log'!J5:J503,"Pass")+COUNTIFS('Inspection Log'!C5:C503,"2026-07-28",'Inspection Log'!J5:J503,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E31" s="7">
+        <f>COUNTIFS('Inspection Log'!C5:C503,"2026-07-28",'Inspection Log'!J5:J503,"Pass")</f>
+        <v/>
+      </c>
+      <c r="F31" s="70">
+        <f>IF(B31="","",IFERROR(C31/B31,0))</f>
+        <v/>
+      </c>
+      <c r="G31" s="70">
+        <f>IF(B31="","",IFERROR(E31/B31,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="62" t="inlineStr">
+        <is>
+          <t>Tech reject % = discarded / received.   Good-from-pit % = IQC good / received (the true end-to-end yield).   IQC good / IQC inspected = the agreement on kept blocks (headline above).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A5:B7"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A10:G10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>